<commit_message>
Top level SV files, and Daily Log complete
Created top level SV files, and PM_DM files, and completed daily log for 5-28
</commit_message>
<xml_diff>
--- a/RISC-V_CST.xlsx
+++ b/RISC-V_CST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Apex\Projects\RISC-V_Project\sfm_RISC-V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99272C05-E342-49CF-8F51-60BD955EA587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7C3C8B-66B4-465E-A7A8-AE3FCEECB894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="45972" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -588,7 +588,7 @@
         <v>32</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>33</v>
@@ -759,7 +759,7 @@
         <v>33</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>33</v>

</xml_diff>